<commit_message>
Fix MEP threshold, upd report files and refactor
v1.14.0

- modelos de reporte con logo 2025
- refact de codigo en el proceso de leer gps
- encriptador actualizado a como estaba en la v2
- tiene el bug de cambio de grados de coordenadas, pero se puede reiniciar manualmente y continuar
</commit_message>
<xml_diff>
--- a/Rastreador GPS+Maps/Resources/Modelo_averif.xlsx
+++ b/Rastreador GPS+Maps/Resources/Modelo_averif.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>Indice</t>
   </si>
@@ -83,6 +83,9 @@
   </si>
   <si>
     <t>MaxHold manual c/incert V/m</t>
+  </si>
+  <si>
+    <t>“2025, Año de la Reconstrucción de la Nación Argentina”</t>
   </si>
 </sst>
 </file>
@@ -127,11 +130,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
+      <name val="Courier New"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -212,11 +214,11 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -237,39 +239,33 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>7619</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>10128</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>798315</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>114300</xdr:rowOff>
+      <xdr:colOff>66675</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>6368</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="3 Imagen"/>
+        <xdr:cNvPr id="5" name="4 Imagen"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="7619" y="10128"/>
-          <a:ext cx="2459476" cy="538512"/>
+          <a:off x="0" y="0"/>
+          <a:ext cx="1733550" cy="1149368"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -589,28 +585,30 @@
     <col min="17" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="13.9" x14ac:dyDescent="0.2">
-      <c r="P1" s="8"/>
+    <row r="1" spans="1:16" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="P1" s="9" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" spans="1:16" ht="18" x14ac:dyDescent="0.2">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
-      <c r="H7" s="9"/>
-      <c r="I7" s="9"/>
-      <c r="J7" s="9"/>
-      <c r="K7" s="9"/>
-      <c r="L7" s="9"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="9"/>
-      <c r="O7" s="9"/>
-      <c r="P7" s="9"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="8"/>
+      <c r="D7" s="8"/>
+      <c r="E7" s="8"/>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8"/>
+      <c r="H7" s="8"/>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
     </row>
     <row r="8" spans="1:16" s="2" customFormat="1" ht="10.9" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="9" spans="1:16" s="2" customFormat="1" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">

</xml_diff>